<commit_message>
Update events: 2026-09-24 18:56 UTC
</commit_message>
<xml_diff>
--- a/docs/events.xlsx
+++ b/docs/events.xlsx
@@ -29881,7 +29881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30218,93 +30218,93 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/26/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>8:30 AM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>USC VS UCLA</t>
+          <t>Rose Bowl Turkey Trot</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
+          <t>https://www.rosebowlstadium.com/events/details/677/rose-bowl-turkey-trot</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/13/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>5:00 AM</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ROSE BOWL FLEA MARKET</t>
+          <t>USC VS UCLA</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
+          <t>https://www.rosebowlstadium.com/events/details/631/usc-vs-ucla</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/13/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>5:00 AM</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>ROSE BOWL FLEA MARKET</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/607/rose-bowl-flea-market</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -30319,19 +30319,19 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/484/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>12/28/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -30346,61 +30346,61 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/485/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01/01/2027</t>
+          <t>12/28/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Rose Bowl Game</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/667/rose-bowl-game</t>
+          <t>https://www.rosebowlstadium.com/events/details/486/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>01/01/2027</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HOLIDAY TOURS</t>
+          <t>Rose Bowl Game</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
+          <t>https://www.rosebowlstadium.com/events/details/667/rose-bowl-game</t>
         </is>
       </c>
     </row>
@@ -30417,56 +30417,56 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10:00 PM</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>HOLIDAY HUDDLE</t>
+          <t>HOLIDAY TOURS</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/668/holiday-huddle</t>
+          <t>https://www.rosebowlstadium.com/events/details/487/holiday-tours</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sunday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01/17/2027</t>
+          <t>01/02/2027</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>10:00 PM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rose Bowl Half Marathon &amp; 5K</t>
+          <t>HOLIDAY HUDDLE</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
+          <t>https://www.rosebowlstadium.com/events/details/668/holiday-huddle</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Sunday</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>04/23/2027</t>
+          <t>01/17/2027</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -30476,24 +30476,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Harry Styles - Together, Together Tour</t>
+          <t>Rose Bowl Half Marathon &amp; 5K</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/673/harry-styles-together-together-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/626/rose-bowl-half-marathon-and-5k</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Saturday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04/24/2027</t>
+          <t>04/23/2027</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -30508,19 +30508,19 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/674/harry-styles-together-together-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/673/harry-styles-together-together-tour</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04/30/2027</t>
+          <t>04/24/2027</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -30530,37 +30530,64 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>HARRY STYLES - TOGETHER, TOGETHER TOUR</t>
+          <t>Harry Styles - Together, Together Tour</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.rosebowlstadium.com/events/details/675/harry-styles-together-together-tour</t>
+          <t>https://www.rosebowlstadium.com/events/details/674/harry-styles-together-together-tour</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>04/30/2027</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>HARRY STYLES - TOGETHER, TOGETHER TOUR</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rosebowlstadium.com/events/details/675/harry-styles-together-together-tour</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Saturday</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>05/01/2027</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>HARRY STYLES - TOGETHER, TOGETHER TOUR</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>https://www.rosebowlstadium.com/events/details/676/harry-styles-together-together-tour</t>
         </is>
@@ -30592,6 +30619,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>